<commit_message>
Leads: 2026-10-29 05:15 UTC (cycle 4)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-29.xlsx
+++ b/output/leads_2026-10-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -563,6 +563,62 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Garland Hot Water Heater</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>waterheatersgarland.com</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://www.waterheatersgarland.com/</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>service@waterheatersgarland.com</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>469-977-2996</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Garland TX</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>water heater repair Garland TX</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-29 05:18 UTC (cycle 6)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-29.xlsx
+++ b/output/leads_2026-10-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -584,7 +584,6 @@
           <t>https://www.waterheatersgarland.com/</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>service@waterheatersgarland.com</t>
@@ -614,6 +613,122 @@
         </is>
       </c>
       <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Valdivia Roofing</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>valdiviaroofing.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://valdiviaroofing.com/service-area/salinas</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Valdivia Roofing</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>humberto@valdiviaroofing.com</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>(408) 940-2162</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Salinas CA</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>90</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>roof replacement Salinas CA</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Roofing Contractor in Ona &amp; Huntington, WV</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>j3roofingwv.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://j3roofingwv.com/</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>j3roofingwv@gmail.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>(304) 397-0550</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Huntington WV</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>88</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>roofing contractor Huntington WV</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
         <is>
           <t>2026-10-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-29 05:20 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-29.xlsx
+++ b/output/leads_2026-10-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -699,7 +699,6 @@
           <t>https://j3roofingwv.com/</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>j3roofingwv@gmail.com</t>
@@ -729,6 +728,66 @@
         </is>
       </c>
       <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Air Conditioning Repair in Long Beach, CA</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>internationalhvacla.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://www.internationalhvacla.com/air-conditioning-repair.html</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Long Beach</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>info@internationalhvacla.com</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>(424) 901-0349</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Long Beach CA</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>90</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>air conditioning repair Long Beach CA</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
         <is>
           <t>2026-10-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-29 05:21 UTC (cycle 8)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-29.xlsx
+++ b/output/leads_2026-10-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -793,6 +793,66 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Graham Plumbing and Drain Cleaning</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>grahamplumbing.net</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://grahamplumbing.net/service-areas/anaheim-ca/drain-cleaning-anaheim-ca</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Overview Why</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>grahamplumbinginc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>(714) 367-4996</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Anaheim CA</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>drain cleaning service Anaheim CA</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-29 05:24 UTC (cycle 10)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-29.xlsx
+++ b/output/leads_2026-10-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -853,6 +853,66 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Peak Home Performance Heating, Air, Plumbing &amp; Electrical</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>gowithpeak.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://gowithpeak.com/areas-served/pueblo/</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Truly Dedicated</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>info@gowithpeak.com</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>(719) 888-5705</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Pueblo CO</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>100</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>HVAC contractor Pueblo CO</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-29 05:26 UTC (cycle 11)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-29.xlsx
+++ b/output/leads_2026-10-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -913,6 +913,62 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Expert Plumbing &amp; Drain Cleaning Services in Fresno and Clovis, CA | Leedway Plu</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>leedwayplumbinginc.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://www.leedwayplumbinginc.com/</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>drainspecialist@att.net</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>559-706-1091</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Fresno CA</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>100</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>drain cleaning service Fresno CA</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-29 15:19 UTC (cycle 11)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-29.xlsx
+++ b/output/leads_2026-10-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -934,7 +934,6 @@
           <t>https://www.leedwayplumbinginc.com/</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>drainspecialist@att.net</t>
@@ -964,6 +963,66 @@
         </is>
       </c>
       <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Sila</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>dcmdva.sila.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://dcmdva.sila.com/hvac-services/heating/heat-pump/</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Round Home</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>webresponse-md@sila.com</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>(240) 301-3846</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Washington DC</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>90</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>heat pump installation Washington DC</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
         <is>
           <t>2026-10-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-29 20:57 UTC (cycle 1)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-29.xlsx
+++ b/output/leads_2026-10-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1028,6 +1028,66 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Brooklyn Roof Repair</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>brooklynroof.repair</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://brooklynroof.repair/</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Work That</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>info@brooklynroof.repair</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>347-298-2236</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Brooklyn NY</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>90</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>roof repair company Brooklyn NY</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-29 21:00 UTC (cycle 3)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-29.xlsx
+++ b/output/leads_2026-10-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1088,6 +1088,62 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Roofing Columbus, GA</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>caldwells-roofing.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://caldwells-roofing.com/roofing-columbus-ga/</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>caldwbr@gmail.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>334-332-7799</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Columbus GA</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>74</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>roofer Columbus GA</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-29 21:06 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-29.xlsx
+++ b/output/leads_2026-10-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1109,7 +1109,6 @@
           <t>https://caldwells-roofing.com/roofing-columbus-ga/</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>caldwbr@gmail.com</t>
@@ -1139,6 +1138,66 @@
         </is>
       </c>
       <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Next Level Pipe Lining</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>nextlevelpipelining.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://nextlevelpipelining.com/service-areas/raleigh-nc/sewer-repair-raleigh-nc/</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>North Carolina</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>info@nextlevelpipelining.com</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>(980) 355-2356</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Raleigh NC</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>90</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>sewer repair Raleigh NC</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
         <is>
           <t>2026-10-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-29 21:08 UTC (cycle 8)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-29.xlsx
+++ b/output/leads_2026-10-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1203,6 +1203,66 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Emergency Plumber in Beaverton, OR | 24/7 Service</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>beavertonplumbingguys.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://beavertonplumbingguys.com/</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Areas Beaverton</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>contact@beavertonplumbingguys.com</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>(971) 326-9890</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Beaverton OR</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>90</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>emergency plumber Beaverton OR</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-29 21:11 UTC (cycle 10)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-29.xlsx
+++ b/output/leads_2026-10-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1263,6 +1263,66 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Accord Air</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>accordair.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://accordair.com/ac/escondido/</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Require Air</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>ahomeshvac@gmail.com</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>858-208-8140</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Escondido CA</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>90</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>AC installation Escondido CA</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>